<commit_message>
Minor imporvements (v. 0.4.3).
</commit_message>
<xml_diff>
--- a/AIMeRiC/corpus/validacio/comparison.xlsx
+++ b/AIMeRiC/corpus/validacio/comparison.xlsx
@@ -447,10 +447,10 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>25.10204081632653</v>
+        <v>25</v>
       </c>
       <c r="B2" t="n">
-        <v>25.10204081632653</v>
+        <v>25</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
@@ -458,13 +458,13 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>64.79591836734694</v>
+        <v>64.89795918367346</v>
       </c>
       <c r="B3" t="n">
         <v>65.10204081632654</v>
       </c>
       <c r="C3" t="n">
-        <v>0.3061224489795933</v>
+        <v>0.2040816326530717</v>
       </c>
     </row>
     <row r="4">
@@ -513,21 +513,21 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>33.16326530612245</v>
+        <v>33.26530612244898</v>
       </c>
       <c r="B8" t="n">
         <v>33.36734693877551</v>
       </c>
       <c r="C8" t="n">
-        <v>0.2040816326530646</v>
+        <v>0.1020408163265358</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
+        <v>64.08163265306122</v>
+      </c>
+      <c r="B9" t="n">
         <v>64.18367346938776</v>
-      </c>
-      <c r="B9" t="n">
-        <v>64.08163265306122</v>
       </c>
       <c r="C9" t="n">
         <v>0.1020408163265358</v>
@@ -538,10 +538,10 @@
         <v>4.387755102040816</v>
       </c>
       <c r="B10" t="n">
-        <v>3.877551020408163</v>
+        <v>4.081632653061225</v>
       </c>
       <c r="C10" t="n">
-        <v>0.510204081632653</v>
+        <v>0.3061224489795915</v>
       </c>
     </row>
     <row r="11">

</xml_diff>

<commit_message>
Actualització en la representació de paraules i síl·labes (emmagatzematge més complet al JSON)
</commit_message>
<xml_diff>
--- a/AIMeRiC/corpus/validacio/comparison.xlsx
+++ b/AIMeRiC/corpus/validacio/comparison.xlsx
@@ -1,54 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr defaultThemeVersion="124226"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
-  <si>
-    <t>Automàtic</t>
-  </si>
-  <si>
-    <t>Manual</t>
-  </si>
-  <si>
-    <t>Diferència</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -63,35 +46,93 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -379,132 +420,142 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Automàtic</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Diferència</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>0.2510204081632653</v>
+      </c>
+      <c r="B2" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.001020408163265318</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>0.6489795918367347</v>
+      </c>
+      <c r="B3" t="n">
+        <v>0.6510204081632653</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.002040816326530637</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>0.1683673469387755</v>
+      </c>
+      <c r="B4" t="n">
+        <v>0.1653061224489796</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.0030612244897959</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>0.9061224489795918</v>
+      </c>
+      <c r="B5" t="n">
+        <v>0.9081632653061225</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.002040816326530637</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>0.05816326530612245</v>
+      </c>
+      <c r="B6" t="n">
+        <v>0.05612244897959184</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.002040816326530609</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>0.7214285714285714</v>
+      </c>
+      <c r="B7" t="n">
+        <v>0.7255102040816327</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.004081632653061273</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>0.336734693877551</v>
+      </c>
+      <c r="B8" t="n">
+        <v>0.3336734693877551</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.0030612244897959</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>0.6397959183673469</v>
+      </c>
+      <c r="B9" t="n">
+        <v>0.6418367346938776</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.002040816326530637</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>0.04387755102040816</v>
+      </c>
+      <c r="B10" t="n">
+        <v>0.04081632653061224</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.00306122448979592</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>1</v>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" t="n">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2">
-        <v>0.25</v>
-      </c>
-      <c r="B2">
-        <v>0.25</v>
-      </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3">
-        <v>0.6489795918367347</v>
-      </c>
-      <c r="B3">
-        <v>0.6510204081632653</v>
-      </c>
-      <c r="C3">
-        <v>0.002040816326530637</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4">
-        <v>0.1673469387755102</v>
-      </c>
-      <c r="B4">
-        <v>0.1653061224489796</v>
-      </c>
-      <c r="C4">
-        <v>0.002040816326530609</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="A5">
-        <v>0.9061224489795918</v>
-      </c>
-      <c r="B5">
-        <v>0.9081632653061225</v>
-      </c>
-      <c r="C5">
-        <v>0.002040816326530637</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
-      <c r="A6">
-        <v>0.05816326530612245</v>
-      </c>
-      <c r="B6">
-        <v>0.05612244897959184</v>
-      </c>
-      <c r="C6">
-        <v>0.002040816326530609</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
-      <c r="A7">
-        <v>0.7244897959183674</v>
-      </c>
-      <c r="B7">
-        <v>0.7255102040816327</v>
-      </c>
-      <c r="C7">
-        <v>0.001020408163265318</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="A8">
-        <v>0.3326530612244898</v>
-      </c>
-      <c r="B8">
-        <v>0.3336734693877551</v>
-      </c>
-      <c r="C8">
-        <v>0.001020408163265318</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
-      <c r="A9">
-        <v>0.6408163265306123</v>
-      </c>
-      <c r="B9">
-        <v>0.6418367346938776</v>
-      </c>
-      <c r="C9">
-        <v>0.001020408163265318</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3">
-      <c r="A10">
-        <v>0.04387755102040816</v>
-      </c>
-      <c r="B10">
-        <v>0.04081632653061224</v>
-      </c>
-      <c r="C10">
-        <v>0.00306122448979592</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3">
-      <c r="A11">
-        <v>1</v>
-      </c>
-      <c r="B11">
-        <v>1</v>
-      </c>
-      <c r="C11">
-        <v>0</v>
-      </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[CONTROL] Actualització de la gestió de patrons en l'etiquetatge de prosa: substitució de 'comparative_pattern' per 'contorn_cru' i eliminació de funcions obsoletes per simplificar el codi.
</commit_message>
<xml_diff>
--- a/AIMeRiC/corpus/validacio/comparison.xlsx
+++ b/AIMeRiC/corpus/validacio/comparison.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -447,43 +447,43 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.2510204081632653</v>
+        <v>0.3295918367346939</v>
       </c>
       <c r="B2" t="n">
-        <v>0.25</v>
+        <v>0.3295918367346939</v>
       </c>
       <c r="C2" t="n">
-        <v>0.001020408163265318</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.6489795918367347</v>
+        <v>0.6530612244897959</v>
       </c>
       <c r="B3" t="n">
-        <v>0.6510204081632653</v>
+        <v>0.6540816326530612</v>
       </c>
       <c r="C3" t="n">
-        <v>0.002040816326530637</v>
+        <v>0.001020408163265318</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.1683673469387755</v>
+        <v>0.09591836734693877</v>
       </c>
       <c r="B4" t="n">
-        <v>0.1653061224489796</v>
+        <v>0.09387755102040816</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0030612244897959</v>
+        <v>0.002040816326530609</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0.9061224489795918</v>
+        <v>0.8989795918367347</v>
       </c>
       <c r="B5" t="n">
-        <v>0.9081632653061225</v>
+        <v>0.9010204081632653</v>
       </c>
       <c r="C5" t="n">
         <v>0.002040816326530637</v>
@@ -491,57 +491,57 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.05816326530612245</v>
+        <v>0.1061224489795918</v>
       </c>
       <c r="B6" t="n">
-        <v>0.05612244897959184</v>
+        <v>0.1051020408163265</v>
       </c>
       <c r="C6" t="n">
-        <v>0.002040816326530609</v>
+        <v>0.001020408163265304</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0.7214285714285714</v>
+        <v>0.6571428571428571</v>
       </c>
       <c r="B7" t="n">
-        <v>0.7255102040816327</v>
+        <v>0.6591836734693878</v>
       </c>
       <c r="C7" t="n">
-        <v>0.004081632653061273</v>
+        <v>0.002040816326530637</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0.336734693877551</v>
+        <v>0.3214285714285715</v>
       </c>
       <c r="B8" t="n">
-        <v>0.3336734693877551</v>
+        <v>0.3214285714285715</v>
       </c>
       <c r="C8" t="n">
-        <v>0.0030612244897959</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0.6397959183673469</v>
+        <v>0.6479591836734694</v>
       </c>
       <c r="B9" t="n">
-        <v>0.6418367346938776</v>
+        <v>0.6489795918367347</v>
       </c>
       <c r="C9" t="n">
-        <v>0.002040816326530637</v>
+        <v>0.001020408163265318</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0.04387755102040816</v>
+        <v>0</v>
       </c>
       <c r="B10" t="n">
-        <v>0.04081632653061224</v>
+        <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>0.00306122448979592</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">

</xml_diff>

<commit_message>
Millores en la gestió de síl·labes i actualitzacions en el mòdul de validació: ajustaments en la identificació de pronoms enclítics, reindexació de síl·labes, i optimització de la funció de tall en versos decasíl·labs.
</commit_message>
<xml_diff>
--- a/AIMeRiC/corpus/validacio/comparison.xlsx
+++ b/AIMeRiC/corpus/validacio/comparison.xlsx
@@ -447,29 +447,29 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.3295918367346939</v>
+        <v>0.3255102040816327</v>
       </c>
       <c r="B2" t="n">
         <v>0.3295918367346939</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>0.004081632653061218</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.6530612244897959</v>
+        <v>0.6561224489795918</v>
       </c>
       <c r="B3" t="n">
         <v>0.6540816326530612</v>
       </c>
       <c r="C3" t="n">
-        <v>0.001020408163265318</v>
+        <v>0.002040816326530637</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.09591836734693877</v>
+        <v>0.09183673469387756</v>
       </c>
       <c r="B4" t="n">
         <v>0.09387755102040816</v>
@@ -480,57 +480,57 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0.8989795918367347</v>
+        <v>0.9051020408163265</v>
       </c>
       <c r="B5" t="n">
         <v>0.9010204081632653</v>
       </c>
       <c r="C5" t="n">
-        <v>0.002040816326530637</v>
+        <v>0.004081632653061162</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.1061224489795918</v>
+        <v>0.03469387755102041</v>
       </c>
       <c r="B6" t="n">
         <v>0.1051020408163265</v>
       </c>
       <c r="C6" t="n">
-        <v>0.001020408163265304</v>
+        <v>0.07040816326530612</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0.6571428571428571</v>
+        <v>0.676530612244898</v>
       </c>
       <c r="B7" t="n">
         <v>0.6591836734693878</v>
       </c>
       <c r="C7" t="n">
-        <v>0.002040816326530637</v>
+        <v>0.01734693877551019</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0.3214285714285715</v>
+        <v>0.3081632653061224</v>
       </c>
       <c r="B8" t="n">
         <v>0.3214285714285715</v>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>0.01326530612244903</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0.6479591836734694</v>
+        <v>0.6561224489795918</v>
       </c>
       <c r="B9" t="n">
         <v>0.6489795918367347</v>
       </c>
       <c r="C9" t="n">
-        <v>0.001020408163265318</v>
+        <v>0.007142857142857117</v>
       </c>
     </row>
     <row r="10">

</xml_diff>

<commit_message>
Actualització de la funció d'etiquetatge: afegit paràmetre 'goal' per personalitzar el mode d'etiquetatge i millorar la flexibilitat en l'anàlisi de corpus.
</commit_message>
<xml_diff>
--- a/AIMeRiC/corpus/validacio/comparison.xlsx
+++ b/AIMeRiC/corpus/validacio/comparison.xlsx
@@ -480,57 +480,57 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0.9051020408163265</v>
+        <v>0.9061224489795918</v>
       </c>
       <c r="B5" t="n">
         <v>0.9010204081632653</v>
       </c>
       <c r="C5" t="n">
-        <v>0.004081632653061162</v>
+        <v>0.005102040816326481</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.03469387755102041</v>
+        <v>0.02857142857142857</v>
       </c>
       <c r="B6" t="n">
         <v>0.1051020408163265</v>
       </c>
       <c r="C6" t="n">
-        <v>0.07040816326530612</v>
+        <v>0.07653061224489796</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0.676530612244898</v>
+        <v>0.6795918367346939</v>
       </c>
       <c r="B7" t="n">
         <v>0.6591836734693878</v>
       </c>
       <c r="C7" t="n">
-        <v>0.01734693877551019</v>
+        <v>0.02040816326530615</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0.3081632653061224</v>
+        <v>0.3061224489795918</v>
       </c>
       <c r="B8" t="n">
         <v>0.3214285714285715</v>
       </c>
       <c r="C8" t="n">
-        <v>0.01326530612244903</v>
+        <v>0.01530612244897961</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0.6561224489795918</v>
+        <v>0.6571428571428571</v>
       </c>
       <c r="B9" t="n">
         <v>0.6489795918367347</v>
       </c>
       <c r="C9" t="n">
-        <v>0.007142857142857117</v>
+        <v>0.008163265306122436</v>
       </c>
     </row>
     <row r="10">

</xml_diff>

<commit_message>
Reajustament de l'accent secundari en mots amb sinèresi.
</commit_message>
<xml_diff>
--- a/AIMeRiC/corpus/validacio/comparison.xlsx
+++ b/AIMeRiC/corpus/validacio/comparison.xlsx
@@ -447,24 +447,24 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.3255102040816327</v>
+        <v>0.2806122448979592</v>
       </c>
       <c r="B2" t="n">
         <v>0.3295918367346939</v>
       </c>
       <c r="C2" t="n">
-        <v>0.004081632653061218</v>
+        <v>0.04897959183673473</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.6551020408163265</v>
+        <v>0.6561224489795918</v>
       </c>
       <c r="B3" t="n">
         <v>0.6540816326530612</v>
       </c>
       <c r="C3" t="n">
-        <v>0.001020408163265318</v>
+        <v>0.002040816326530637</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
Afegit script de diagnòstic per a la funció `tall()` i millores en la gestió de talls mètrics; inclou proves per a la subdivisió i validacions de condicions
</commit_message>
<xml_diff>
--- a/AIMeRiC/corpus/validacio/comparison.xlsx
+++ b/AIMeRiC/corpus/validacio/comparison.xlsx
@@ -447,90 +447,90 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.2744897959183674</v>
+        <v>0.2724489795918367</v>
       </c>
       <c r="B2" t="n">
         <v>0.3295918367346939</v>
       </c>
       <c r="C2" t="n">
-        <v>0.05510204081632653</v>
+        <v>0.05714285714285716</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.6540816326530612</v>
+        <v>0.6479591836734694</v>
       </c>
       <c r="B3" t="n">
         <v>0.6540816326530612</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>0.006122448979591799</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.09285714285714286</v>
+        <v>0.1071428571428571</v>
       </c>
       <c r="B4" t="n">
         <v>0.09387755102040816</v>
       </c>
       <c r="C4" t="n">
-        <v>0.001020408163265304</v>
+        <v>0.01326530612244897</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0.9051020408163265</v>
+        <v>0.8877551020408163</v>
       </c>
       <c r="B5" t="n">
         <v>0.9010204081632653</v>
       </c>
       <c r="C5" t="n">
-        <v>0.004081632653061162</v>
+        <v>0.01326530612244903</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.03061224489795918</v>
+        <v>0.03877551020408163</v>
       </c>
       <c r="B6" t="n">
         <v>0.1051020408163265</v>
       </c>
       <c r="C6" t="n">
-        <v>0.07448979591836735</v>
+        <v>0.06632653061224489</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0.686734693877551</v>
+        <v>0.6857142857142857</v>
       </c>
       <c r="B7" t="n">
         <v>0.6591836734693878</v>
       </c>
       <c r="C7" t="n">
-        <v>0.02755102040816326</v>
+        <v>0.02653061224489794</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0.3081632653061224</v>
+        <v>0.3071428571428572</v>
       </c>
       <c r="B8" t="n">
         <v>0.3214285714285715</v>
       </c>
       <c r="C8" t="n">
-        <v>0.01326530612244903</v>
+        <v>0.01428571428571429</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0.6846938775510204</v>
+        <v>0.686734693877551</v>
       </c>
       <c r="B9" t="n">
         <v>0.6489795918367347</v>
       </c>
       <c r="C9" t="n">
-        <v>0.0357142857142857</v>
+        <v>0.03775510204081634</v>
       </c>
     </row>
     <row r="10">

</xml_diff>

<commit_message>
Millores en la gestió de la conversió de dades a CSV; afegida gestió d'errors i forçada la conversió de columnes a cadenes. Safety check aplicat a còlons.
</commit_message>
<xml_diff>
--- a/AIMeRiC/corpus/validacio/comparison.xlsx
+++ b/AIMeRiC/corpus/validacio/comparison.xlsx
@@ -447,24 +447,24 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.2724489795918367</v>
+        <v>0.2673469387755102</v>
       </c>
       <c r="B2" t="n">
         <v>0.3295918367346939</v>
       </c>
       <c r="C2" t="n">
-        <v>0.05714285714285716</v>
+        <v>0.0622448979591837</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.6479591836734694</v>
+        <v>0.6530612244897959</v>
       </c>
       <c r="B3" t="n">
         <v>0.6540816326530612</v>
       </c>
       <c r="C3" t="n">
-        <v>0.006122448979591799</v>
+        <v>0.001020408163265318</v>
       </c>
     </row>
     <row r="4">
@@ -480,57 +480,57 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0.8877551020408163</v>
+        <v>0.8908163265306123</v>
       </c>
       <c r="B5" t="n">
         <v>0.9010204081632653</v>
       </c>
       <c r="C5" t="n">
-        <v>0.01326530612244903</v>
+        <v>0.01020408163265307</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.03877551020408163</v>
+        <v>0.03571428571428571</v>
       </c>
       <c r="B6" t="n">
         <v>0.1051020408163265</v>
       </c>
       <c r="C6" t="n">
-        <v>0.06632653061224489</v>
+        <v>0.06938775510204082</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0.6857142857142857</v>
+        <v>0.6836734693877551</v>
       </c>
       <c r="B7" t="n">
         <v>0.6591836734693878</v>
       </c>
       <c r="C7" t="n">
-        <v>0.02653061224489794</v>
+        <v>0.02448979591836731</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0.3071428571428572</v>
+        <v>0.3061224489795918</v>
       </c>
       <c r="B8" t="n">
         <v>0.3214285714285715</v>
       </c>
       <c r="C8" t="n">
-        <v>0.01428571428571429</v>
+        <v>0.01530612244897961</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0.686734693877551</v>
+        <v>0.6887755102040817</v>
       </c>
       <c r="B9" t="n">
         <v>0.6489795918367347</v>
       </c>
       <c r="C9" t="n">
-        <v>0.03775510204081634</v>
+        <v>0.03979591836734697</v>
       </c>
     </row>
     <row r="10">

</xml_diff>